<commit_message>
feat: switch PRODOC evaluation rubric to sustainability assessment file
- Changed rubric source from PRODOC_rubric.xlsx to Evaluación de sostenibilidad del proyecto_rubric_7nov.xlsx
- Updated binary rubric file with new sustainability evaluation criteria
- Commented out previous PRODOC rubric loading line for reference
</commit_message>
<xml_diff>
--- a/Evaluación de sostenibilidad del proyecto_rubric_7nov.xlsx
+++ b/Evaluación de sostenibilidad del proyecto_rubric_7nov.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bezzolo\Desktop\3ra. sesión\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ageidv/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC57121-EB3B-4DE0-B0FF-B76F0E99E751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4507A909-50B3-4947-A9A2-CE03B9B50C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Diseño" sheetId="1" r:id="rId1"/>
+    <sheet name="rubric" sheetId="1" r:id="rId1"/>
     <sheet name="Implementación" sheetId="4" r:id="rId2"/>
     <sheet name="Evaluación" sheetId="5" r:id="rId3"/>
   </sheets>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="133">
   <si>
     <t>Criterio</t>
   </si>
@@ -3530,12 +3530,24 @@
       <t xml:space="preserve"> para llevar a cabo las políticas, planes, estrategias y actividades necesarias para consolidar los resultados de la intervención.</t>
     </r>
   </si>
+  <si>
+    <t>Dimensión</t>
+  </si>
+  <si>
+    <t>Diseño</t>
+  </si>
+  <si>
+    <t>Evaluación</t>
+  </si>
+  <si>
+    <t>Implementación</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3681,7 +3693,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3721,6 +3733,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3917,153 +3932,909 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="28.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.54296875" style="2" customWidth="1"/>
-    <col min="3" max="6" width="60" style="2" customWidth="1"/>
-    <col min="16384" max="16384" width="11.54296875" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5" style="2" customWidth="1"/>
+    <col min="4" max="7" width="60" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" ht="16">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="143" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:7" ht="154">
+      <c r="A2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="208" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:7" ht="224">
+      <c r="A3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="119" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:7" ht="119" customHeight="1">
+      <c r="A4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="234" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:7" ht="238">
+      <c r="A5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="143" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:7" ht="140">
+      <c r="A6" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="260" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:7" ht="252">
+      <c r="A7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="45" customHeight="1">
+      <c r="A18" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="52" customHeight="1">
+      <c r="A19" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A20" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A21" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A22" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A23" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A24" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A25" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A26" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A27" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A28" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A29" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A30" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A31" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A32" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A33" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A34" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A35" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A36" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A37" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A38" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="12.75" customHeight="1">
+      <c r="A39" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -4078,235 +4849,268 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{020B241B-7BE5-483E-846F-051555D35178}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="28.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="70.81640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="69.36328125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="65.90625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="74.08984375" style="2" customWidth="1"/>
-    <col min="16384" max="16384" width="11.54296875" customWidth="1"/>
+    <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="65.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="74.1640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" ht="16">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="180.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:7" ht="180.5" customHeight="1">
+      <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="117" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:7" ht="112">
+      <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="192" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:7" ht="192" customHeight="1">
+      <c r="A4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="78" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:7" ht="84">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="177" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:7" ht="177" customHeight="1">
+      <c r="A6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="178" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:7" ht="178" customHeight="1">
+      <c r="A7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="260.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:7" ht="260.5" customHeight="1">
+      <c r="A8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="D8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="E8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="F8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="G8" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="248.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:7" ht="248.5" customHeight="1">
+      <c r="A9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="185.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:7" ht="185.5" customHeight="1">
+      <c r="A10" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="282" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:7" ht="282" customHeight="1">
+      <c r="A11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4322,475 +5126,543 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EC5BE52-010A-4C15-80F1-1D67C4485BA8}">
-  <dimension ref="A1:F23"/>
-  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="28.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.54296875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="70.81640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="69.36328125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="65.90625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="74.08984375" style="2" customWidth="1"/>
-    <col min="16384" max="16384" width="11.54296875" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="65.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="74.1640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" ht="16">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="143" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:7" ht="140">
+      <c r="A2" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="195" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:7" ht="196">
+      <c r="A3" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="153.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:7" ht="153.5" customHeight="1">
+      <c r="A4" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="180.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:7" ht="180.5" customHeight="1">
+      <c r="A5" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="117" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:7" ht="112">
+      <c r="A6" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="208" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:7" ht="224">
+      <c r="A7" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="130" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:7" ht="126">
+      <c r="A8" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="260.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:7" ht="260.5" customHeight="1">
+      <c r="A9" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="F9" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="338.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:7" ht="338.5" customHeight="1">
+      <c r="A10" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="D10" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="E10" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="G10" s="11" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="260" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:7" ht="252">
+      <c r="A11" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="248.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+    <row r="12" spans="1:7" ht="248.5" customHeight="1">
+      <c r="A12" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="185.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:7" ht="185.5" customHeight="1">
+      <c r="A13" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="289" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:7" ht="289" customHeight="1">
+      <c r="A14" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="192" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+    <row r="15" spans="1:7" ht="192" customHeight="1">
+      <c r="A15" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="D15" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="E15" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="F15" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="G15" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="78" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:7" ht="84">
+      <c r="A16" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="C16" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="177" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:7" ht="177" customHeight="1">
+      <c r="A17" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="178" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:7" ht="178" customHeight="1">
+      <c r="A18" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="192" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:7" ht="192" customHeight="1">
+      <c r="A19" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="D19" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="E19" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="F19" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="G19" s="8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="179" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:7" ht="179" customHeight="1">
+      <c r="A20" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="C20" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="D20" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="E20" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="F20" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="G20" s="8" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="178" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:7" ht="178" customHeight="1">
+      <c r="A21" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="C21" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="282" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:7" ht="282" customHeight="1">
+      <c r="A22" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="178" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:7" ht="178" customHeight="1">
+      <c r="A23" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="C23" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: rename 'Evaluación' dimension to 'Pre-Cierre' in deployment configuration.
</commit_message>
<xml_diff>
--- a/Evaluación de sostenibilidad del proyecto_rubric_7nov.xlsx
+++ b/Evaluación de sostenibilidad del proyecto_rubric_7nov.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ageidv/ilo/deploy_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE502CE-5E91-8747-8EDC-27A8CD2916DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E2AA26-A9D2-7B4A-B4BE-FD2150EFA77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="134">
   <si>
     <t>Criterio</t>
   </si>
@@ -3541,6 +3541,9 @@
   </si>
   <si>
     <t>Implementación</t>
+  </si>
+  <si>
+    <t>Pre-Cierre</t>
   </si>
 </sst>
 </file>
@@ -3693,7 +3696,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3737,7 +3740,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3771,7 +3773,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3970,907 +3972,906 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="11.5" style="15"/>
-    <col min="2" max="2" width="28.5" style="27" customWidth="1"/>
+    <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5" style="26" customWidth="1"/>
     <col min="3" max="3" width="28.5" style="2" customWidth="1"/>
     <col min="4" max="7" width="60" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="11.5" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:7" ht="14">
+      <c r="A1" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:7" ht="14">
+      <c r="A2" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="19" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:7" ht="14">
+      <c r="A3" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:7" ht="14">
+      <c r="A4" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:7" ht="14">
+      <c r="A5" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:7" ht="14">
+      <c r="A6" t="s">
         <v>130</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15">
-      <c r="A7" s="15" t="s">
+    <row r="7" spans="1:7" ht="14">
+      <c r="A7" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:7" ht="14">
+      <c r="A8" t="s">
         <v>132</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="19" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:7" ht="14">
+      <c r="A9" t="s">
         <v>132</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="19" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:7" ht="14">
+      <c r="A10" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="15">
-      <c r="A11" s="15" t="s">
+    <row r="11" spans="1:7" ht="14">
+      <c r="A11" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15">
-      <c r="A12" s="15" t="s">
+    <row r="12" spans="1:7" ht="14">
+      <c r="A12" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="F12" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15">
-      <c r="A13" s="15" t="s">
+    <row r="13" spans="1:7" ht="14">
+      <c r="A13" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>117</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="G13" s="19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:7" ht="14">
+      <c r="A14" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="15">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:7" ht="14">
+      <c r="A15" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="15">
-      <c r="A16" s="15" t="s">
+    <row r="16" spans="1:7" ht="14">
+      <c r="A16" t="s">
         <v>132</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="G16" s="19" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15">
-      <c r="A17" s="15" t="s">
+    <row r="17" spans="1:7" ht="14">
+      <c r="A17" t="s">
         <v>132</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="20" t="s">
+      <c r="E17" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G17" s="19" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15">
+    <row r="18" spans="1:7" ht="14">
       <c r="A18" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B18" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C18" s="19" t="s">
+      <c r="C18" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="19" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15">
+    <row r="19" spans="1:7" ht="14">
       <c r="A19" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B19" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G19" s="19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15">
+    <row r="20" spans="1:7" ht="14">
       <c r="A20" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B20" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="19" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15">
+    <row r="21" spans="1:7" ht="14">
       <c r="A21" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B21" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="F21" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="19" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15">
+    <row r="22" spans="1:7" ht="14">
       <c r="A22" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B22" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F22" s="20" t="s">
+      <c r="F22" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="19" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15">
+    <row r="23" spans="1:7" ht="14">
       <c r="A23" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B23" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="F23" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="24" t="s">
+      <c r="G23" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15">
+    <row r="24" spans="1:7" ht="14">
       <c r="A24" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B24" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="F24" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="G24" s="19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15">
+    <row r="25" spans="1:7" ht="14">
       <c r="A25" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B25" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="25" t="s">
+      <c r="E25" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="G25" s="25" t="s">
+      <c r="G25" s="24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15">
+    <row r="26" spans="1:7" ht="14">
       <c r="A26" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B26" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="E26" s="25" t="s">
+      <c r="E26" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="F26" s="25" t="s">
+      <c r="F26" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="25" t="s">
+      <c r="G26" s="24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15">
+    <row r="27" spans="1:7" ht="14">
       <c r="A27" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B27" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="24" t="s">
+      <c r="D27" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="24" t="s">
+      <c r="E27" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="F27" s="24" t="s">
+      <c r="F27" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="G27" s="24" t="s">
+      <c r="G27" s="23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15">
+    <row r="28" spans="1:7" ht="14">
       <c r="A28" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B28" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="D28" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="E28" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F28" s="20" t="s">
+      <c r="F28" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="G28" s="20" t="s">
+      <c r="G28" s="19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15">
+    <row r="29" spans="1:7" ht="14">
       <c r="A29" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B29" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="F29" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="G29" s="19" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15">
+    <row r="30" spans="1:7" ht="14">
       <c r="A30" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B30" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B30" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="C30" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="F30" s="20" t="s">
+      <c r="F30" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="G30" s="19" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15">
+    <row r="31" spans="1:7" ht="14">
       <c r="A31" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B31" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="D31" s="24" t="s">
+      <c r="D31" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E31" s="24" t="s">
+      <c r="E31" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="F31" s="24" t="s">
+      <c r="F31" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="G31" s="24" t="s">
+      <c r="G31" s="23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15">
+    <row r="32" spans="1:7" ht="14">
       <c r="A32" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B32" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C32" s="23" t="s">
+      <c r="C32" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15">
+    <row r="33" spans="1:7" ht="14">
       <c r="A33" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B33" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="C33" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F33" s="20" t="s">
+      <c r="F33" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="19" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15">
+    <row r="34" spans="1:7" ht="14">
       <c r="A34" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B34" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C34" s="23" t="s">
+      <c r="C34" s="22" t="s">
         <v>117</v>
       </c>
-      <c r="D34" s="20" t="s">
+      <c r="D34" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="E34" s="20" t="s">
+      <c r="E34" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="F34" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15">
+    <row r="35" spans="1:7" ht="14">
       <c r="A35" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B35" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="C35" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="D35" s="24" t="s">
+      <c r="D35" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="F35" s="24" t="s">
+      <c r="F35" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="G35" s="24" t="s">
+      <c r="G35" s="23" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="14">
       <c r="A36" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B36" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B36" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="C36" s="23" t="s">
+      <c r="C36" s="22" t="s">
         <v>126</v>
       </c>
-      <c r="D36" s="24" t="s">
+      <c r="D36" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="E36" s="24" t="s">
+      <c r="E36" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="F36" s="24" t="s">
+      <c r="F36" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="G36" s="24" t="s">
+      <c r="G36" s="23" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15">
+    <row r="37" spans="1:7" ht="14">
       <c r="A37" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B37" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C37" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="D37" s="20" t="s">
+      <c r="D37" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="E37" s="20" t="s">
+      <c r="E37" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="F37" s="20" t="s">
+      <c r="F37" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="19" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15">
+    <row r="38" spans="1:7" ht="14">
       <c r="A38" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B38" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B38" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="C38" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="D38" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E38" s="20" t="s">
+      <c r="E38" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F38" s="20" t="s">
+      <c r="F38" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="G38" s="19" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15">
+    <row r="39" spans="1:7" ht="14">
       <c r="A39" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B39" s="26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B39" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="C39" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="E39" s="20" t="s">
+      <c r="E39" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="F39" s="20" t="s">
+      <c r="F39" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="G39" s="19" t="s">
         <v>89</v>
       </c>
     </row>
@@ -4898,7 +4899,7 @@
     <col min="7" max="7" width="74.1640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16">
+    <row r="1" spans="1:7" ht="15">
       <c r="A1" t="s">
         <v>129</v>
       </c>
@@ -5174,7 +5175,7 @@
     <col min="7" max="7" width="74.1640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16">
+    <row r="1" spans="1:7" ht="15">
       <c r="A1" t="s">
         <v>129</v>
       </c>

</xml_diff>